<commit_message>
students and faculty data update
</commit_message>
<xml_diff>
--- a/excels/Phd_Current.xlsx
+++ b/excels/Phd_Current.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\NITW-Transportation-Division-main\NITW-Transportation-Division-main\excels\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\nitw\NITW-Transportation-Division\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{409D45F2-D608-4DA5-A5CF-32294E6EB26E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8663708C-2022-4139-BFE3-57F4C14894F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -273,9 +273,6 @@
     <t>Multi-Modal Development in Transport Planning</t>
   </si>
   <si>
-    <t>https://drive.google.com/uc?export=view&amp;id=1y51fE3wn2025MBIaO7Cox8os7Qc_1G7f</t>
-  </si>
-  <si>
     <t>https://www.nitw.ac.in/CIVDeptAssets/images/phd62.jpg</t>
   </si>
   <si>
@@ -301,6 +298,9 @@
   </si>
   <si>
     <t>shailaja</t>
+  </si>
+  <si>
+    <t>Anjaneyulu</t>
   </si>
 </sst>
 </file>
@@ -719,219 +719,219 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C2" s="5">
-        <v>9492203336</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>17</v>
+        <v>32</v>
+      </c>
+      <c r="B2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C2">
+        <v>9494353643</v>
+      </c>
+      <c r="D2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>83</v>
+        <v>68</v>
+      </c>
+      <c r="B3" s="10">
+        <v>720028</v>
+      </c>
+      <c r="C3">
+        <v>8296368016</v>
+      </c>
+      <c r="D3" t="s">
+        <v>69</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" s="4">
-        <v>8500970790</v>
+        <v>20</v>
+      </c>
+      <c r="C4" s="5">
+        <v>9492203336</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E4" t="s">
-        <v>27</v>
+        <v>19</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>21</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>7</v>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>33</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>34</v>
       </c>
       <c r="C5">
-        <v>9542093078</v>
+        <v>7902240230</v>
       </c>
       <c r="D5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F5" t="s">
-        <v>11</v>
+        <v>37</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" t="s">
-        <v>9</v>
+        <v>43</v>
+      </c>
+      <c r="B6" s="8">
+        <v>701905</v>
       </c>
       <c r="C6">
-        <v>9167519065</v>
+        <v>9502607177</v>
       </c>
       <c r="D6" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F6" t="s">
-        <v>29</v>
+        <v>44</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>31</v>
-      </c>
-      <c r="B7" t="s">
-        <v>85</v>
+        <v>70</v>
+      </c>
+      <c r="B7" s="10">
+        <v>720029</v>
       </c>
       <c r="C7">
-        <v>9381752788</v>
+        <v>7296367016</v>
       </c>
       <c r="D7" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="F7" t="s">
-        <v>91</v>
+        <v>35</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>41</v>
+        <v>9</v>
       </c>
       <c r="C8">
-        <v>9494353643</v>
+        <v>9167519065</v>
       </c>
       <c r="D8" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
-        <v>33</v>
+        <v>10</v>
+      </c>
+      <c r="F8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>31</v>
       </c>
       <c r="B9" t="s">
-        <v>34</v>
+        <v>84</v>
       </c>
       <c r="C9">
-        <v>7902240230</v>
+        <v>9381752788</v>
       </c>
       <c r="D9" t="s">
-        <v>37</v>
+        <v>81</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>39</v>
+        <v>89</v>
+      </c>
+      <c r="F9" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>43</v>
-      </c>
-      <c r="B10" s="8">
-        <v>701905</v>
-      </c>
-      <c r="C10">
-        <v>9502607177</v>
-      </c>
-      <c r="D10" t="s">
-        <v>42</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>45</v>
+        <v>6</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" s="4">
+        <v>8500970790</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E10" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>46</v>
-      </c>
-      <c r="B11" s="10">
-        <v>720018</v>
-      </c>
-      <c r="C11" s="9">
-        <v>9555541646</v>
-      </c>
-      <c r="D11" t="s">
-        <v>47</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>48</v>
+        <v>5</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>50</v>
+        <v>72</v>
       </c>
       <c r="B12" s="10">
-        <v>720019</v>
+        <v>720030</v>
       </c>
       <c r="C12">
-        <v>7386310538</v>
+        <v>6296367016</v>
       </c>
       <c r="D12" t="s">
-        <v>51</v>
+        <v>73</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>87</v>
+        <v>35</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>48</v>
@@ -939,19 +939,19 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B13" s="10">
-        <v>720020</v>
+        <v>720019</v>
       </c>
       <c r="C13">
-        <v>8639717077</v>
+        <v>7386310538</v>
       </c>
       <c r="D13" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>48</v>
@@ -959,36 +959,36 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>54</v>
-      </c>
-      <c r="B14" s="10">
-        <v>720021</v>
+        <v>7</v>
+      </c>
+      <c r="B14" t="s">
+        <v>12</v>
       </c>
       <c r="C14">
-        <v>9381442621</v>
+        <v>9542093078</v>
       </c>
       <c r="D14" t="s">
-        <v>55</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>48</v>
+        <v>28</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F14" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B15" s="10">
-        <v>720022</v>
+        <v>720021</v>
       </c>
       <c r="C15">
-        <v>8296369017</v>
+        <v>9381442621</v>
       </c>
       <c r="D15" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>35</v>
@@ -999,19 +999,19 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="B16" s="10">
-        <v>720023</v>
+        <v>720020</v>
       </c>
       <c r="C16">
-        <v>8296369016</v>
+        <v>8639717077</v>
       </c>
       <c r="D16" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>35</v>
+        <v>87</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>48</v>
@@ -1019,16 +1019,16 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="B17" s="10">
-        <v>720024</v>
+        <v>720022</v>
       </c>
       <c r="C17">
-        <v>8294367016</v>
+        <v>8296369017</v>
       </c>
       <c r="D17" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>35</v>
@@ -1039,36 +1039,36 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>62</v>
-      </c>
-      <c r="B18" s="10">
-        <v>720025</v>
+        <v>74</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>83</v>
       </c>
       <c r="C18">
-        <v>8236367016</v>
+        <v>9032426878</v>
       </c>
       <c r="D18" t="s">
-        <v>63</v>
+        <v>75</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>35</v>
+        <v>88</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>48</v>
+        <v>91</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="B19" s="10">
-        <v>720026</v>
+        <v>720023</v>
       </c>
       <c r="C19">
-        <v>8196367016</v>
+        <v>8296369016</v>
       </c>
       <c r="D19" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>35</v>
@@ -1079,16 +1079,16 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="B20" s="10">
-        <v>720027</v>
+        <v>720025</v>
       </c>
       <c r="C20">
-        <v>8296367116</v>
+        <v>8236367016</v>
       </c>
       <c r="D20" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>35</v>
@@ -1099,16 +1099,16 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="B21" s="10">
-        <v>720028</v>
+        <v>720024</v>
       </c>
       <c r="C21">
-        <v>8296368016</v>
+        <v>8294367016</v>
       </c>
       <c r="D21" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>35</v>
@@ -1119,16 +1119,16 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="B22" s="10">
-        <v>720029</v>
+        <v>720032</v>
       </c>
       <c r="C22">
-        <v>7296367016</v>
+        <v>9296367016</v>
       </c>
       <c r="D22" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>35</v>
@@ -1139,16 +1139,16 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="B23" s="10">
-        <v>720030</v>
+        <v>720026</v>
       </c>
       <c r="C23">
-        <v>6296367016</v>
+        <v>8196367016</v>
       </c>
       <c r="D23" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>35</v>
@@ -1159,36 +1159,36 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>74</v>
-      </c>
-      <c r="B24" s="10" t="s">
-        <v>84</v>
-      </c>
-      <c r="C24">
-        <v>9032426878</v>
+        <v>46</v>
+      </c>
+      <c r="B24" s="10">
+        <v>720018</v>
+      </c>
+      <c r="C24" s="9">
+        <v>9555541646</v>
       </c>
       <c r="D24" t="s">
-        <v>75</v>
+        <v>47</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>89</v>
+        <v>49</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>82</v>
+        <v>48</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="B25" s="10">
-        <v>720032</v>
+        <v>720027</v>
       </c>
       <c r="C25">
-        <v>9296367016</v>
+        <v>8296367116</v>
       </c>
       <c r="D25" t="s">
-        <v>86</v>
+        <v>67</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>35</v>
@@ -1199,16 +1199,16 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B26" s="10">
-        <v>720033</v>
+        <v>720034</v>
       </c>
       <c r="C26">
-        <v>8295367016</v>
+        <v>8286367016</v>
       </c>
       <c r="D26" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>35</v>
@@ -1219,16 +1219,16 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B27" s="10">
-        <v>720034</v>
+        <v>720033</v>
       </c>
       <c r="C27">
-        <v>8286367016</v>
+        <v>8295367016</v>
       </c>
       <c r="D27" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>35</v>
@@ -1238,53 +1238,55 @@
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F27">
+    <sortCondition ref="A2:A27"/>
+  </sortState>
   <hyperlinks>
-    <hyperlink ref="E6" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="E5" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="F4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="F2" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="E8" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="E9" r:id="rId6" display="mailto:aa23cer1r01@student.nitw.ac.in" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="F9" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="F8" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="E10" r:id="rId9" display="mailto:so701905@student.nitw.ac.in" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="F11" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="F10" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="E11" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="E7" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="E12" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="E13" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
-    <hyperlink ref="E14" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="E15" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="E16" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="E17" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="E18" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
-    <hyperlink ref="E19" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
-    <hyperlink ref="E20" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
-    <hyperlink ref="E21" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
-    <hyperlink ref="E22" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
-    <hyperlink ref="E23" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
-    <hyperlink ref="E24" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
-    <hyperlink ref="E25" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
-    <hyperlink ref="E26" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
-    <hyperlink ref="E27" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
-    <hyperlink ref="F12" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
-    <hyperlink ref="F13" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
-    <hyperlink ref="F14" r:id="rId32" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
-    <hyperlink ref="F15" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
-    <hyperlink ref="F16" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
-    <hyperlink ref="F17" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
-    <hyperlink ref="F18" r:id="rId36" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
-    <hyperlink ref="F19" r:id="rId37" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
-    <hyperlink ref="F20" r:id="rId38" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
-    <hyperlink ref="F21" r:id="rId39" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
-    <hyperlink ref="F22" r:id="rId40" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
-    <hyperlink ref="F23" r:id="rId41" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
-    <hyperlink ref="F24" r:id="rId42" xr:uid="{00000000-0004-0000-0000-000029000000}"/>
-    <hyperlink ref="F25" r:id="rId43" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
-    <hyperlink ref="F26" r:id="rId44" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
-    <hyperlink ref="F27" r:id="rId45" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
-    <hyperlink ref="F3" r:id="rId46" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
+    <hyperlink ref="E8" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="E14" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="F10" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="F4" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="E2" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="E5" r:id="rId6" display="mailto:aa23cer1r01@student.nitw.ac.in" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="F5" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="F2" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="E6" r:id="rId9" display="mailto:so701905@student.nitw.ac.in" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="F24" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="F6" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="E24" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="E9" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="E13" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="E16" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="E15" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="E17" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="E19" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="E21" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="E20" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="E23" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="E25" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="E3" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="E7" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="E12" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="E18" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="E22" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="E27" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
+    <hyperlink ref="E26" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
+    <hyperlink ref="F13" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
+    <hyperlink ref="F16" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
+    <hyperlink ref="F15" r:id="rId32" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
+    <hyperlink ref="F17" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
+    <hyperlink ref="F19" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
+    <hyperlink ref="F21" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
+    <hyperlink ref="F20" r:id="rId36" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
+    <hyperlink ref="F23" r:id="rId37" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
+    <hyperlink ref="F25" r:id="rId38" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
+    <hyperlink ref="F3" r:id="rId39" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
+    <hyperlink ref="F7" r:id="rId40" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
+    <hyperlink ref="F12" r:id="rId41" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
+    <hyperlink ref="F22" r:id="rId42" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
+    <hyperlink ref="F27" r:id="rId43" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
+    <hyperlink ref="F26" r:id="rId44" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
+    <hyperlink ref="F11" r:id="rId45" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
updated vision, mission and scholor data
</commit_message>
<xml_diff>
--- a/excels/Phd_Current.xlsx
+++ b/excels/Phd_Current.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\nitw\NITW-Transportation-Division\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8663708C-2022-4139-BFE3-57F4C14894F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A397EA5A-DAF6-4E7B-92B7-E4A0CE23CCA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="96">
   <si>
     <t xml:space="preserve">Name </t>
   </si>
@@ -301,6 +301,18 @@
   </si>
   <si>
     <t>Anjaneyulu</t>
+  </si>
+  <si>
+    <t>Gullapelly Mounika</t>
+  </si>
+  <si>
+    <t>25CER1R08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Traffic Flow Modelling and Simulation </t>
+  </si>
+  <si>
+    <t>gm25cer1r08@student.nitw.ac.in</t>
   </si>
 </sst>
 </file>
@@ -684,7 +696,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.140625" customWidth="1"/>
@@ -959,59 +971,56 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>7</v>
+        <v>92</v>
       </c>
       <c r="B14" t="s">
-        <v>12</v>
+        <v>93</v>
       </c>
       <c r="C14">
-        <v>9542093078</v>
+        <v>9951815536</v>
       </c>
       <c r="D14" t="s">
-        <v>28</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F14" t="s">
-        <v>11</v>
+        <v>94</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>54</v>
-      </c>
-      <c r="B15" s="10">
-        <v>720021</v>
+        <v>7</v>
+      </c>
+      <c r="B15" t="s">
+        <v>12</v>
       </c>
       <c r="C15">
-        <v>9381442621</v>
+        <v>9542093078</v>
       </c>
       <c r="D15" t="s">
-        <v>55</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>48</v>
+        <v>28</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B16" s="10">
-        <v>720020</v>
+        <v>720021</v>
       </c>
       <c r="C16">
-        <v>8639717077</v>
+        <v>9381442621</v>
       </c>
       <c r="D16" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>87</v>
+        <v>35</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>48</v>
@@ -1019,19 +1028,19 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="B17" s="10">
-        <v>720022</v>
+        <v>720020</v>
       </c>
       <c r="C17">
-        <v>8296369017</v>
+        <v>8639717077</v>
       </c>
       <c r="D17" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>35</v>
+        <v>87</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>48</v>
@@ -1039,56 +1048,56 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>74</v>
-      </c>
-      <c r="B18" s="10" t="s">
-        <v>83</v>
+        <v>56</v>
+      </c>
+      <c r="B18" s="10">
+        <v>720022</v>
       </c>
       <c r="C18">
-        <v>9032426878</v>
+        <v>8296369017</v>
       </c>
       <c r="D18" t="s">
-        <v>75</v>
+        <v>57</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>88</v>
+        <v>35</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>91</v>
+        <v>48</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>58</v>
-      </c>
-      <c r="B19" s="10">
-        <v>720023</v>
+        <v>74</v>
+      </c>
+      <c r="B19" s="10" t="s">
+        <v>83</v>
       </c>
       <c r="C19">
-        <v>8296369016</v>
+        <v>9032426878</v>
       </c>
       <c r="D19" t="s">
-        <v>59</v>
+        <v>75</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>35</v>
+        <v>88</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>48</v>
+        <v>91</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B20" s="10">
-        <v>720025</v>
+        <v>720023</v>
       </c>
       <c r="C20">
-        <v>8236367016</v>
+        <v>8296369016</v>
       </c>
       <c r="D20" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>35</v>
@@ -1099,16 +1108,16 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B21" s="10">
-        <v>720024</v>
+        <v>720025</v>
       </c>
       <c r="C21">
-        <v>8294367016</v>
+        <v>8236367016</v>
       </c>
       <c r="D21" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>35</v>
@@ -1119,16 +1128,16 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>76</v>
+        <v>60</v>
       </c>
       <c r="B22" s="10">
-        <v>720032</v>
+        <v>720024</v>
       </c>
       <c r="C22">
-        <v>9296367016</v>
+        <v>8294367016</v>
       </c>
       <c r="D22" t="s">
-        <v>85</v>
+        <v>61</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>35</v>
@@ -1139,16 +1148,16 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>64</v>
+        <v>76</v>
       </c>
       <c r="B23" s="10">
-        <v>720026</v>
+        <v>720032</v>
       </c>
       <c r="C23">
-        <v>8196367016</v>
+        <v>9296367016</v>
       </c>
       <c r="D23" t="s">
-        <v>65</v>
+        <v>85</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>35</v>
@@ -1159,19 +1168,19 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>46</v>
+        <v>64</v>
       </c>
       <c r="B24" s="10">
-        <v>720018</v>
-      </c>
-      <c r="C24" s="9">
-        <v>9555541646</v>
+        <v>720026</v>
+      </c>
+      <c r="C24">
+        <v>8196367016</v>
       </c>
       <c r="D24" t="s">
-        <v>47</v>
+        <v>65</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>48</v>
@@ -1179,19 +1188,19 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>66</v>
+        <v>46</v>
       </c>
       <c r="B25" s="10">
-        <v>720027</v>
-      </c>
-      <c r="C25">
-        <v>8296367116</v>
+        <v>720018</v>
+      </c>
+      <c r="C25" s="9">
+        <v>9555541646</v>
       </c>
       <c r="D25" t="s">
-        <v>67</v>
+        <v>47</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>35</v>
+        <v>49</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>48</v>
@@ -1199,16 +1208,16 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>79</v>
+        <v>66</v>
       </c>
       <c r="B26" s="10">
-        <v>720034</v>
+        <v>720027</v>
       </c>
       <c r="C26">
-        <v>8286367016</v>
+        <v>8296367116</v>
       </c>
       <c r="D26" t="s">
-        <v>80</v>
+        <v>67</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>35</v>
@@ -1219,16 +1228,16 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B27" s="10">
-        <v>720033</v>
+        <v>720034</v>
       </c>
       <c r="C27">
-        <v>8295367016</v>
+        <v>8286367016</v>
       </c>
       <c r="D27" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>35</v>
@@ -1237,13 +1246,33 @@
         <v>48</v>
       </c>
     </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>77</v>
+      </c>
+      <c r="B28" s="10">
+        <v>720033</v>
+      </c>
+      <c r="C28">
+        <v>8295367016</v>
+      </c>
+      <c r="D28" t="s">
+        <v>78</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F27">
-    <sortCondition ref="A2:A27"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F28">
+    <sortCondition ref="A27:A28"/>
   </sortState>
   <hyperlinks>
     <hyperlink ref="E8" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="E14" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="E15" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
     <hyperlink ref="F10" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
     <hyperlink ref="F4" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
     <hyperlink ref="E2" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
@@ -1251,42 +1280,43 @@
     <hyperlink ref="F5" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
     <hyperlink ref="F2" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
     <hyperlink ref="E6" r:id="rId9" display="mailto:so701905@student.nitw.ac.in" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="F24" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="F25" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
     <hyperlink ref="F6" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="E24" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="E25" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
     <hyperlink ref="E9" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
     <hyperlink ref="E13" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="E16" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
-    <hyperlink ref="E15" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="E17" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="E19" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="E21" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="E20" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
-    <hyperlink ref="E23" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
-    <hyperlink ref="E25" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="E17" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="E16" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="E18" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="E20" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="E22" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="E21" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="E24" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="E26" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
     <hyperlink ref="E3" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
     <hyperlink ref="E7" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
     <hyperlink ref="E12" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
-    <hyperlink ref="E18" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
-    <hyperlink ref="E22" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
-    <hyperlink ref="E27" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
-    <hyperlink ref="E26" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
+    <hyperlink ref="E19" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="E23" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="E28" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
+    <hyperlink ref="E27" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
     <hyperlink ref="F13" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
-    <hyperlink ref="F16" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
-    <hyperlink ref="F15" r:id="rId32" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
-    <hyperlink ref="F17" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
-    <hyperlink ref="F19" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
-    <hyperlink ref="F21" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
-    <hyperlink ref="F20" r:id="rId36" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
-    <hyperlink ref="F23" r:id="rId37" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
-    <hyperlink ref="F25" r:id="rId38" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
+    <hyperlink ref="F17" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
+    <hyperlink ref="F16" r:id="rId32" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
+    <hyperlink ref="F18" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
+    <hyperlink ref="F20" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
+    <hyperlink ref="F22" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
+    <hyperlink ref="F21" r:id="rId36" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
+    <hyperlink ref="F24" r:id="rId37" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
+    <hyperlink ref="F26" r:id="rId38" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
     <hyperlink ref="F3" r:id="rId39" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
     <hyperlink ref="F7" r:id="rId40" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
     <hyperlink ref="F12" r:id="rId41" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
-    <hyperlink ref="F22" r:id="rId42" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
-    <hyperlink ref="F27" r:id="rId43" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
-    <hyperlink ref="F26" r:id="rId44" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
+    <hyperlink ref="F23" r:id="rId42" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
+    <hyperlink ref="F28" r:id="rId43" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
+    <hyperlink ref="F27" r:id="rId44" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
     <hyperlink ref="F11" r:id="rId45" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
+    <hyperlink ref="E14" r:id="rId46" xr:uid="{CBA56252-7528-480E-896E-AE82E42DF951}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
updates on socialmedia links, logo image
</commit_message>
<xml_diff>
--- a/excels/Phd_Current.xlsx
+++ b/excels/Phd_Current.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\nitw\NITW-Transportation-Division\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A397EA5A-DAF6-4E7B-92B7-E4A0CE23CCA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8969821A-EE20-44C0-9F72-A750B4C13C67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rs" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="95">
   <si>
     <t xml:space="preserve">Name </t>
   </si>
@@ -169,9 +169,6 @@
   </si>
   <si>
     <t>Travel Behaviour with Built Environment Characteristics</t>
-  </si>
-  <si>
-    <t>https://www.nitw.ac.in/CIVDeptAssets/images/phd38.jpg</t>
   </si>
   <si>
     <t>ckumarcivil@gmail.com</t>
@@ -751,7 +748,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B3" s="10">
         <v>720028</v>
@@ -760,14 +757,12 @@
         <v>8296368016</v>
       </c>
       <c r="D3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="F3" s="2" t="s">
-        <v>48</v>
-      </c>
+      <c r="F3" s="2"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
@@ -831,7 +826,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B7" s="10">
         <v>720029</v>
@@ -840,14 +835,12 @@
         <v>7296367016</v>
       </c>
       <c r="D7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="F7" s="2" t="s">
-        <v>48</v>
-      </c>
+      <c r="F7" s="2"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
@@ -874,19 +867,19 @@
         <v>31</v>
       </c>
       <c r="B9" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C9">
         <v>9381752788</v>
       </c>
       <c r="D9" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E9" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="F9" t="s">
         <v>89</v>
-      </c>
-      <c r="F9" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -926,12 +919,12 @@
         <v>25</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B12" s="10">
         <v>720030</v>
@@ -940,18 +933,16 @@
         <v>6296367016</v>
       </c>
       <c r="D12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="F12" s="2" t="s">
-        <v>48</v>
-      </c>
+      <c r="F12" s="2"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B13" s="10">
         <v>720019</v>
@@ -960,30 +951,28 @@
         <v>7386310538</v>
       </c>
       <c r="D13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>48</v>
-      </c>
+        <v>85</v>
+      </c>
+      <c r="F13" s="2"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>91</v>
+      </c>
+      <c r="B14" t="s">
         <v>92</v>
-      </c>
-      <c r="B14" t="s">
-        <v>93</v>
       </c>
       <c r="C14">
         <v>9951815536</v>
       </c>
       <c r="D14" t="s">
+        <v>93</v>
+      </c>
+      <c r="E14" s="2" t="s">
         <v>94</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -1008,7 +997,7 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B16" s="10">
         <v>720021</v>
@@ -1017,18 +1006,16 @@
         <v>9381442621</v>
       </c>
       <c r="D16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="F16" s="2" t="s">
-        <v>48</v>
-      </c>
+      <c r="F16" s="2"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B17" s="10">
         <v>720020</v>
@@ -1037,18 +1024,16 @@
         <v>8639717077</v>
       </c>
       <c r="D17" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>48</v>
-      </c>
+        <v>86</v>
+      </c>
+      <c r="F17" s="2"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B18" s="10">
         <v>720022</v>
@@ -1057,38 +1042,36 @@
         <v>8296369017</v>
       </c>
       <c r="D18" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="F18" s="2" t="s">
-        <v>48</v>
-      </c>
+      <c r="F18" s="2"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C19">
         <v>9032426878</v>
       </c>
       <c r="D19" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B20" s="10">
         <v>720023</v>
@@ -1097,18 +1080,16 @@
         <v>8296369016</v>
       </c>
       <c r="D20" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="F20" s="2" t="s">
-        <v>48</v>
-      </c>
+      <c r="F20" s="2"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B21" s="10">
         <v>720025</v>
@@ -1117,18 +1098,16 @@
         <v>8236367016</v>
       </c>
       <c r="D21" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="F21" s="2" t="s">
-        <v>48</v>
-      </c>
+      <c r="F21" s="2"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B22" s="10">
         <v>720024</v>
@@ -1137,18 +1116,16 @@
         <v>8294367016</v>
       </c>
       <c r="D22" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="F22" s="2" t="s">
-        <v>48</v>
-      </c>
+      <c r="F22" s="2"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B23" s="10">
         <v>720032</v>
@@ -1157,18 +1134,16 @@
         <v>9296367016</v>
       </c>
       <c r="D23" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="F23" s="2" t="s">
-        <v>48</v>
-      </c>
+      <c r="F23" s="2"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B24" s="10">
         <v>720026</v>
@@ -1177,14 +1152,12 @@
         <v>8196367016</v>
       </c>
       <c r="D24" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="F24" s="2" t="s">
-        <v>48</v>
-      </c>
+      <c r="F24" s="2"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
@@ -1200,15 +1173,13 @@
         <v>47</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="F25" s="2" t="s">
         <v>48</v>
       </c>
+      <c r="F25" s="2"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B26" s="10">
         <v>720027</v>
@@ -1217,18 +1188,16 @@
         <v>8296367116</v>
       </c>
       <c r="D26" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="F26" s="2" t="s">
-        <v>48</v>
-      </c>
+      <c r="F26" s="2"/>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B27" s="10">
         <v>720034</v>
@@ -1237,18 +1206,16 @@
         <v>8286367016</v>
       </c>
       <c r="D27" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="F27" s="2" t="s">
-        <v>48</v>
-      </c>
+      <c r="F27" s="2"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B28" s="10">
         <v>720033</v>
@@ -1257,14 +1224,12 @@
         <v>8295367016</v>
       </c>
       <c r="D28" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="F28" s="2" t="s">
-        <v>48</v>
-      </c>
+      <c r="F28" s="2"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F28">
@@ -1280,43 +1245,27 @@
     <hyperlink ref="F5" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
     <hyperlink ref="F2" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
     <hyperlink ref="E6" r:id="rId9" display="mailto:so701905@student.nitw.ac.in" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="F25" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="F6" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="E25" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="E9" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="E13" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="E17" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
-    <hyperlink ref="E16" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="E18" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="E20" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="E22" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="E21" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
-    <hyperlink ref="E24" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
-    <hyperlink ref="E26" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
-    <hyperlink ref="E3" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
-    <hyperlink ref="E7" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
-    <hyperlink ref="E12" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
-    <hyperlink ref="E19" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
-    <hyperlink ref="E23" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
-    <hyperlink ref="E28" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
-    <hyperlink ref="E27" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
-    <hyperlink ref="F13" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
-    <hyperlink ref="F17" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
-    <hyperlink ref="F16" r:id="rId32" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
-    <hyperlink ref="F18" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
-    <hyperlink ref="F20" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
-    <hyperlink ref="F22" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
-    <hyperlink ref="F21" r:id="rId36" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
-    <hyperlink ref="F24" r:id="rId37" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
-    <hyperlink ref="F26" r:id="rId38" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
-    <hyperlink ref="F3" r:id="rId39" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
-    <hyperlink ref="F7" r:id="rId40" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
-    <hyperlink ref="F12" r:id="rId41" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
-    <hyperlink ref="F23" r:id="rId42" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
-    <hyperlink ref="F28" r:id="rId43" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
-    <hyperlink ref="F27" r:id="rId44" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
-    <hyperlink ref="F11" r:id="rId45" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
-    <hyperlink ref="E14" r:id="rId46" xr:uid="{CBA56252-7528-480E-896E-AE82E42DF951}"/>
+    <hyperlink ref="F6" r:id="rId10" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="E25" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="E9" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="E18" r:id="rId13" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="E20" r:id="rId14" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="E22" r:id="rId15" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="E21" r:id="rId16" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="E24" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="E26" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="E19" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="E23" r:id="rId20" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="E28" r:id="rId21" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
+    <hyperlink ref="E27" r:id="rId22" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
+    <hyperlink ref="F11" r:id="rId23" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
+    <hyperlink ref="E14" r:id="rId24" xr:uid="{CBA56252-7528-480E-896E-AE82E42DF951}"/>
+    <hyperlink ref="E17" r:id="rId25" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="E16" r:id="rId26" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="E13" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="E12" r:id="rId28" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="E7" r:id="rId29" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="E3" r:id="rId30" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
updates as per suggestions
</commit_message>
<xml_diff>
--- a/excels/Phd_Current.xlsx
+++ b/excels/Phd_Current.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\nitw\NITW-Transportation-Division\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8969821A-EE20-44C0-9F72-A750B4C13C67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AB11F59-51FB-42B3-B5E5-62FAF182385E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rs" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="96">
   <si>
     <t xml:space="preserve">Name </t>
   </si>
@@ -310,6 +310,9 @@
   </si>
   <si>
     <t>gm25cer1r08@student.nitw.ac.in</t>
+  </si>
+  <si>
+    <t>mounika</t>
   </si>
 </sst>
 </file>
@@ -974,6 +977,9 @@
       <c r="E14" s="2" t="s">
         <v>94</v>
       </c>
+      <c r="F14" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">

</xml_diff>

<commit_message>
updated publication design and phd scholars study mode
</commit_message>
<xml_diff>
--- a/excels/Phd_Current.xlsx
+++ b/excels/Phd_Current.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\nitw\NITW-Transportation-Division\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AB11F59-51FB-42B3-B5E5-62FAF182385E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6099ABD7-CF4F-4A03-B731-C451D0AAC642}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="99">
   <si>
     <t xml:space="preserve">Name </t>
   </si>
@@ -93,9 +93,6 @@
     <t>as21cerer13@student.nitw.ac.in</t>
   </si>
   <si>
-    <t>21CEFJ005</t>
-  </si>
-  <si>
     <t> 9993290666</t>
   </si>
   <si>
@@ -313,6 +310,18 @@
   </si>
   <si>
     <t>mounika</t>
+  </si>
+  <si>
+    <t>21CEFJ005/712005</t>
+  </si>
+  <si>
+    <t>Study Mode</t>
+  </si>
+  <si>
+    <t>Full Time</t>
+  </si>
+  <si>
+    <t>Part Time</t>
   </si>
 </sst>
 </file>
@@ -389,7 +398,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
@@ -405,15 +414,17 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -696,10 +707,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="29.140625" customWidth="1"/>
+    <col min="1" max="1" width="29.140625" style="11" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
     <col min="3" max="3" width="19.42578125" customWidth="1"/>
     <col min="4" max="4" width="57.5703125" customWidth="1"/>
@@ -709,8 +720,8 @@
     <col min="10" max="10" width="22.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -728,47 +739,56 @@
       <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>32</v>
+      <c r="G1" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="11" t="s">
+        <v>31</v>
       </c>
       <c r="B2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C2">
         <v>9494353643</v>
       </c>
       <c r="D2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>67</v>
-      </c>
-      <c r="B3" s="10">
+        <v>39</v>
+      </c>
+      <c r="G2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="B3" s="9">
         <v>720028</v>
       </c>
       <c r="C3">
         <v>8296368016</v>
       </c>
       <c r="D3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F3" s="2"/>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="G3" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="11" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="4" t="s">
@@ -786,67 +806,79 @@
       <c r="F4" s="3" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
+      <c r="G4" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A5" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" t="s">
         <v>33</v>
-      </c>
-      <c r="B5" t="s">
-        <v>34</v>
       </c>
       <c r="C5">
         <v>7902240230</v>
       </c>
       <c r="D5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="F5" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="F5" s="2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>43</v>
-      </c>
-      <c r="B6" s="8">
+      <c r="G5" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" s="7">
         <v>701905</v>
       </c>
       <c r="C6">
         <v>9502607177</v>
       </c>
       <c r="D6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E6" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="F6" s="2" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>69</v>
-      </c>
-      <c r="B7" s="10">
+      <c r="G6" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="B7" s="9">
         <v>720029</v>
       </c>
       <c r="C7">
         <v>7296367016</v>
       </c>
       <c r="D7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F7" s="2"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="G7" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="11" t="s">
         <v>8</v>
       </c>
       <c r="B8" t="s">
@@ -856,37 +888,43 @@
         <v>9167519065</v>
       </c>
       <c r="D8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F8" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>31</v>
+        <v>28</v>
+      </c>
+      <c r="G8" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="11" t="s">
+        <v>30</v>
       </c>
       <c r="B9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C9">
         <v>9381752788</v>
       </c>
       <c r="D9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E9" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="F9" t="s">
         <v>88</v>
       </c>
-      <c r="F9" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="G9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="11" t="s">
         <v>6</v>
       </c>
       <c r="B10" s="4" t="s">
@@ -896,93 +934,108 @@
         <v>8500970790</v>
       </c>
       <c r="D10" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E10" t="s">
         <v>26</v>
-      </c>
-      <c r="E10" t="s">
-        <v>27</v>
       </c>
       <c r="F10" s="3" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="G10" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="11" t="s">
         <v>5</v>
       </c>
       <c r="B11" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="C11" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="D11" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="E11" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="E11" s="5" t="s">
-        <v>25</v>
-      </c>
       <c r="F11" s="3" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>71</v>
-      </c>
-      <c r="B12" s="10">
+        <v>80</v>
+      </c>
+      <c r="G11" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="B12" s="9">
         <v>720030</v>
       </c>
       <c r="C12">
         <v>6296367016</v>
       </c>
       <c r="D12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F12" s="2"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>49</v>
-      </c>
-      <c r="B13" s="10">
+      <c r="G12" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="B13" s="9">
         <v>720019</v>
       </c>
       <c r="C13">
         <v>7386310538</v>
       </c>
       <c r="D13" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F13" s="2"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+      <c r="G13" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="B14" t="s">
         <v>91</v>
-      </c>
-      <c r="B14" t="s">
-        <v>92</v>
       </c>
       <c r="C14">
         <v>9951815536</v>
       </c>
       <c r="D14" t="s">
+        <v>92</v>
+      </c>
+      <c r="E14" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="F14" t="s">
         <v>94</v>
       </c>
-      <c r="F14" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+      <c r="G14" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="11" t="s">
         <v>7</v>
       </c>
       <c r="B15" t="s">
@@ -992,7 +1045,7 @@
         <v>9542093078</v>
       </c>
       <c r="D15" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>13</v>
@@ -1000,242 +1053,284 @@
       <c r="F15" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>53</v>
-      </c>
-      <c r="B16" s="10">
+      <c r="G15" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="B16" s="9">
         <v>720021</v>
       </c>
       <c r="C16">
         <v>9381442621</v>
       </c>
       <c r="D16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F16" s="2"/>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>51</v>
-      </c>
-      <c r="B17" s="10">
+      <c r="G16" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="B17" s="9">
         <v>720020</v>
       </c>
       <c r="C17">
         <v>8639717077</v>
       </c>
       <c r="D17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F17" s="2"/>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>55</v>
-      </c>
-      <c r="B18" s="10">
+      <c r="G17" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="B18" s="9">
         <v>720022</v>
       </c>
       <c r="C18">
         <v>8296369017</v>
       </c>
       <c r="D18" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F18" s="2"/>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>73</v>
-      </c>
-      <c r="B19" s="10" t="s">
-        <v>82</v>
+      <c r="G18" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>81</v>
       </c>
       <c r="C19">
         <v>9032426878</v>
       </c>
       <c r="D19" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>57</v>
-      </c>
-      <c r="B20" s="10">
+        <v>89</v>
+      </c>
+      <c r="G19" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B20" s="9">
         <v>720023</v>
       </c>
       <c r="C20">
         <v>8296369016</v>
       </c>
       <c r="D20" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F20" s="2"/>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>61</v>
-      </c>
-      <c r="B21" s="10">
+      <c r="G20" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="B21" s="9">
         <v>720025</v>
       </c>
       <c r="C21">
         <v>8236367016</v>
       </c>
       <c r="D21" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F21" s="2"/>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>59</v>
-      </c>
-      <c r="B22" s="10">
+      <c r="G21" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="B22" s="9">
         <v>720024</v>
       </c>
       <c r="C22">
         <v>8294367016</v>
       </c>
       <c r="D22" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F22" s="2"/>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>75</v>
-      </c>
-      <c r="B23" s="10">
+      <c r="G22" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="B23" s="9">
         <v>720032</v>
       </c>
       <c r="C23">
         <v>9296367016</v>
       </c>
       <c r="D23" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F23" s="2"/>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>63</v>
-      </c>
-      <c r="B24" s="10">
+      <c r="G23" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="B24" s="9">
         <v>720026</v>
       </c>
       <c r="C24">
         <v>8196367016</v>
       </c>
       <c r="D24" t="s">
+        <v>63</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F24" s="2"/>
+      <c r="G24" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25" s="9">
+        <v>720018</v>
+      </c>
+      <c r="C25" s="8">
+        <v>9555541646</v>
+      </c>
+      <c r="D25" t="s">
+        <v>46</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="F25" s="2"/>
+      <c r="G25" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="E24" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F24" s="2"/>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>46</v>
-      </c>
-      <c r="B25" s="10">
-        <v>720018</v>
-      </c>
-      <c r="C25" s="9">
-        <v>9555541646</v>
-      </c>
-      <c r="D25" t="s">
-        <v>47</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="F25" s="2"/>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>65</v>
-      </c>
-      <c r="B26" s="10">
+      <c r="B26" s="9">
         <v>720027</v>
       </c>
       <c r="C26">
         <v>8296367116</v>
       </c>
       <c r="D26" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F26" s="2"/>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>78</v>
-      </c>
-      <c r="B27" s="10">
+      <c r="G26" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="B27" s="9">
         <v>720034</v>
       </c>
       <c r="C27">
         <v>8286367016</v>
       </c>
       <c r="D27" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F27" s="2"/>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>76</v>
-      </c>
-      <c r="B28" s="10">
+      <c r="G27" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="B28" s="9">
         <v>720033</v>
       </c>
       <c r="C28">
         <v>8295367016</v>
       </c>
       <c r="D28" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F28" s="2"/>
+      <c r="G28" t="s">
+        <v>97</v>
+      </c>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F28">

</xml_diff>

<commit_message>
active button color and current phd images update
</commit_message>
<xml_diff>
--- a/excels/Phd_Current.xlsx
+++ b/excels/Phd_Current.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\nitw\NITW-Transportation-Division\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BFA65DD-838D-4466-B4AD-811BD7C306C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A518498-A5B8-4F58-967E-4D628E5562FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="121">
   <si>
     <t xml:space="preserve">Name </t>
   </si>
@@ -288,12 +288,6 @@
     <t>bs25cer2r13@student.nitw.ac.in</t>
   </si>
   <si>
-    <t>shailaja</t>
-  </si>
-  <si>
-    <t>Anjaneyulu</t>
-  </si>
-  <si>
     <t>Gullapelly Mounika</t>
   </si>
   <si>
@@ -306,9 +300,6 @@
     <t>gm25cer1r08@student.nitw.ac.in</t>
   </si>
   <si>
-    <t>mounika</t>
-  </si>
-  <si>
     <t>21CEFJ005/712005</t>
   </si>
   <si>
@@ -322,13 +313,88 @@
   </si>
   <si>
     <t>Shailaja Bogi</t>
+  </si>
+  <si>
+    <t>25CER2R08</t>
+  </si>
+  <si>
+    <t>yp25cer2r08@student.nitw.ac.in</t>
+  </si>
+  <si>
+    <t>Ammu B C</t>
+  </si>
+  <si>
+    <t>22CER2P01</t>
+  </si>
+  <si>
+    <t>Full depth reclamation mixes</t>
+  </si>
+  <si>
+    <t>ab22cer2p01@student.nitw.ac.in</t>
+  </si>
+  <si>
+    <t>22CER1P10</t>
+  </si>
+  <si>
+    <t>24CER2R05</t>
+  </si>
+  <si>
+    <t>23CER1R18</t>
+  </si>
+  <si>
+    <t>25CER1P07</t>
+  </si>
+  <si>
+    <t>24CER2R06</t>
+  </si>
+  <si>
+    <t>24CER1P02</t>
+  </si>
+  <si>
+    <t>22CER1P08</t>
+  </si>
+  <si>
+    <t>phd_Current/Ammu</t>
+  </si>
+  <si>
+    <t>phd_Current/mounika</t>
+  </si>
+  <si>
+    <t>phd_Current/23CER1R18</t>
+  </si>
+  <si>
+    <t>phd_Current/24CER2R05</t>
+  </si>
+  <si>
+    <t>phd_Current/24CER1P02</t>
+  </si>
+  <si>
+    <t>phd_Current/Anjaneyulu</t>
+  </si>
+  <si>
+    <t>phd_Current/25CER1P07</t>
+  </si>
+  <si>
+    <t>phd_Current/24CER2R06</t>
+  </si>
+  <si>
+    <t>phd_Current/shailaja</t>
+  </si>
+  <si>
+    <t>phd_Current/22CER1P08</t>
+  </si>
+  <si>
+    <t>phd_Current/22CER1P10</t>
+  </si>
+  <si>
+    <t>phd_Current/25CER2R08</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -376,6 +442,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF162C5B"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -398,7 +470,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
@@ -424,6 +496,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -705,7 +778,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.140625" customWidth="1"/>
@@ -738,7 +811,7 @@
         <v>3</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -761,7 +834,7 @@
         <v>38</v>
       </c>
       <c r="G2" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -782,7 +855,7 @@
       </c>
       <c r="F3" s="2"/>
       <c r="G3" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -805,7 +878,7 @@
         <v>17</v>
       </c>
       <c r="G4" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
@@ -828,7 +901,7 @@
         <v>37</v>
       </c>
       <c r="G5" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -851,7 +924,7 @@
         <v>43</v>
       </c>
       <c r="G6" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -872,499 +945,543 @@
       </c>
       <c r="F7" s="2"/>
       <c r="G7" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>8</v>
+        <v>98</v>
       </c>
       <c r="B8" t="s">
-        <v>9</v>
+        <v>99</v>
       </c>
       <c r="C8">
-        <v>9167519065</v>
-      </c>
-      <c r="D8" t="s">
-        <v>29</v>
+        <v>9495307599</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>100</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>10</v>
+        <v>101</v>
       </c>
       <c r="F8" t="s">
-        <v>28</v>
+        <v>109</v>
       </c>
       <c r="G8" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>6</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="C9" s="4">
-        <v>8500970790</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="E9" t="s">
-        <v>26</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>16</v>
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9">
+        <v>9167519065</v>
+      </c>
+      <c r="D9" t="s">
+        <v>29</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F9" t="s">
+        <v>28</v>
       </c>
       <c r="G9" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>5</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>24</v>
+        <v>6</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" s="4">
+        <v>8500970790</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E10" t="s">
+        <v>26</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>79</v>
+        <v>16</v>
       </c>
       <c r="G10" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>69</v>
-      </c>
-      <c r="B11" s="9">
-        <v>720030</v>
-      </c>
-      <c r="C11">
-        <v>6296367016</v>
-      </c>
-      <c r="D11" t="s">
-        <v>70</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="F11" s="2"/>
+        <v>5</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>79</v>
+      </c>
       <c r="G11" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>47</v>
+        <v>69</v>
       </c>
       <c r="B12" s="9">
-        <v>720019</v>
+        <v>720030</v>
       </c>
       <c r="C12">
-        <v>7386310538</v>
+        <v>6296367016</v>
       </c>
       <c r="D12" t="s">
-        <v>48</v>
+        <v>70</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>83</v>
+        <v>33</v>
       </c>
       <c r="F12" s="2"/>
       <c r="G12" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>89</v>
-      </c>
-      <c r="B13" t="s">
-        <v>90</v>
+        <v>47</v>
+      </c>
+      <c r="B13" s="9">
+        <v>720019</v>
       </c>
       <c r="C13">
-        <v>9951815536</v>
+        <v>7386310538</v>
       </c>
       <c r="D13" t="s">
-        <v>91</v>
+        <v>48</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="F13" t="s">
-        <v>93</v>
-      </c>
+        <v>83</v>
+      </c>
+      <c r="F13" s="2"/>
       <c r="G13" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>7</v>
+        <v>87</v>
       </c>
       <c r="B14" t="s">
-        <v>12</v>
+        <v>88</v>
       </c>
       <c r="C14">
-        <v>9542093078</v>
+        <v>9951815536</v>
       </c>
       <c r="D14" t="s">
-        <v>27</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>13</v>
+        <v>89</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>90</v>
       </c>
       <c r="F14" t="s">
-        <v>11</v>
+        <v>110</v>
       </c>
       <c r="G14" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>51</v>
-      </c>
-      <c r="B15" s="9">
-        <v>720021</v>
+        <v>7</v>
+      </c>
+      <c r="B15" t="s">
+        <v>12</v>
       </c>
       <c r="C15">
-        <v>9381442621</v>
+        <v>9542093078</v>
       </c>
       <c r="D15" t="s">
-        <v>52</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="F15" s="2"/>
+        <v>27</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15" t="s">
+        <v>11</v>
+      </c>
       <c r="G15" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>49</v>
-      </c>
-      <c r="B16" s="9">
-        <v>720020</v>
+        <v>51</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>104</v>
       </c>
       <c r="C16">
-        <v>8639717077</v>
+        <v>9381442621</v>
       </c>
       <c r="D16" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="F16" s="2"/>
+        <v>33</v>
+      </c>
+      <c r="F16" t="s">
+        <v>111</v>
+      </c>
       <c r="G16" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>53</v>
-      </c>
-      <c r="B17" s="9">
-        <v>720022</v>
+        <v>49</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>103</v>
       </c>
       <c r="C17">
-        <v>8296369017</v>
+        <v>8639717077</v>
       </c>
       <c r="D17" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="F17" s="2"/>
+        <v>84</v>
+      </c>
+      <c r="F17" t="s">
+        <v>112</v>
+      </c>
       <c r="G17" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>71</v>
+        <v>53</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>80</v>
+        <v>107</v>
       </c>
       <c r="C18">
-        <v>9032426878</v>
+        <v>8296369017</v>
       </c>
       <c r="D18" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>88</v>
+        <v>33</v>
+      </c>
+      <c r="F18" t="s">
+        <v>113</v>
       </c>
       <c r="G18" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>55</v>
-      </c>
-      <c r="B19" s="9">
-        <v>720023</v>
+        <v>71</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>80</v>
       </c>
       <c r="C19">
-        <v>8296369016</v>
+        <v>9032426878</v>
       </c>
       <c r="D19" t="s">
-        <v>56</v>
+        <v>72</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="F19" s="2"/>
+        <v>85</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>114</v>
+      </c>
       <c r="G19" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>59</v>
-      </c>
-      <c r="B20" s="9">
-        <v>720025</v>
+        <v>55</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>105</v>
       </c>
       <c r="C20">
-        <v>8236367016</v>
+        <v>8296369016</v>
       </c>
       <c r="D20" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="F20" s="2"/>
+      <c r="F20" t="s">
+        <v>115</v>
+      </c>
       <c r="G20" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>57</v>
-      </c>
-      <c r="B21" s="9">
-        <v>720024</v>
+        <v>59</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>106</v>
       </c>
       <c r="C21">
-        <v>8294367016</v>
+        <v>8236367016</v>
       </c>
       <c r="D21" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="F21" s="2"/>
+      <c r="F21" t="s">
+        <v>116</v>
+      </c>
       <c r="G21" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>73</v>
+        <v>57</v>
       </c>
       <c r="B22" s="9">
-        <v>720032</v>
+        <v>720024</v>
       </c>
       <c r="C22">
-        <v>9296367016</v>
+        <v>8294367016</v>
       </c>
       <c r="D22" t="s">
-        <v>82</v>
+        <v>58</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>33</v>
       </c>
       <c r="F22" s="2"/>
       <c r="G22" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>98</v>
-      </c>
-      <c r="B23" t="s">
-        <v>81</v>
+        <v>73</v>
+      </c>
+      <c r="B23" s="9">
+        <v>720032</v>
       </c>
       <c r="C23">
-        <v>9381752788</v>
+        <v>9296367016</v>
       </c>
       <c r="D23" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="F23" t="s">
-        <v>87</v>
-      </c>
+        <v>33</v>
+      </c>
+      <c r="F23" s="2"/>
       <c r="G23" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>61</v>
-      </c>
-      <c r="B24" s="9">
-        <v>720026</v>
+        <v>95</v>
+      </c>
+      <c r="B24" t="s">
+        <v>81</v>
       </c>
       <c r="C24">
-        <v>8196367016</v>
+        <v>9381752788</v>
       </c>
       <c r="D24" t="s">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="F24" s="2"/>
+        <v>86</v>
+      </c>
+      <c r="F24" t="s">
+        <v>117</v>
+      </c>
       <c r="G24" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="B25" s="9">
-        <v>720018</v>
-      </c>
-      <c r="C25" s="8">
-        <v>9555541646</v>
+        <v>720026</v>
+      </c>
+      <c r="C25">
+        <v>8196367016</v>
       </c>
       <c r="D25" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>46</v>
+        <v>33</v>
       </c>
       <c r="F25" s="2"/>
       <c r="G25" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>63</v>
+        <v>44</v>
       </c>
       <c r="B26" s="9">
-        <v>720027</v>
-      </c>
-      <c r="C26">
-        <v>8296367116</v>
+        <v>720018</v>
+      </c>
+      <c r="C26" s="8">
+        <v>9555541646</v>
       </c>
       <c r="D26" t="s">
-        <v>64</v>
+        <v>45</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="F26" s="2"/>
       <c r="G26" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>76</v>
-      </c>
-      <c r="B27" s="9">
-        <v>720034</v>
+        <v>63</v>
+      </c>
+      <c r="B27" s="9" t="s">
+        <v>108</v>
       </c>
       <c r="C27">
-        <v>8286367016</v>
+        <v>8296367116</v>
       </c>
       <c r="D27" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="F27" s="2"/>
+      <c r="F27" t="s">
+        <v>118</v>
+      </c>
       <c r="G27" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>74</v>
-      </c>
-      <c r="B28" s="9">
-        <v>720033</v>
+        <v>76</v>
+      </c>
+      <c r="B28" s="9" t="s">
+        <v>102</v>
       </c>
       <c r="C28">
-        <v>8295367016</v>
+        <v>8286367016</v>
       </c>
       <c r="D28" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="F28" s="2"/>
+      <c r="F28" s="2" t="s">
+        <v>119</v>
+      </c>
       <c r="G28" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>74</v>
+      </c>
+      <c r="B29" s="9" t="s">
         <v>96</v>
       </c>
+      <c r="C29">
+        <v>9948673907</v>
+      </c>
+      <c r="D29" t="s">
+        <v>75</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="G29" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D30" s="11"/>
+      <c r="E30" s="2"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G28">
     <sortCondition ref="A12:A28"/>
   </sortState>
   <hyperlinks>
-    <hyperlink ref="E8" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="E14" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="F9" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="E9" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="E15" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="F10" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
     <hyperlink ref="F4" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
     <hyperlink ref="E2" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
     <hyperlink ref="E5" r:id="rId6" display="mailto:aa23cer1r01@student.nitw.ac.in" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
     <hyperlink ref="F5" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
     <hyperlink ref="F2" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
     <hyperlink ref="E6" r:id="rId9" display="mailto:so701905@student.nitw.ac.in" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="F6" r:id="rId10" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="E25" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="E23" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="E17" r:id="rId13" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="E19" r:id="rId14" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="E21" r:id="rId15" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="E20" r:id="rId16" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
-    <hyperlink ref="E24" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
-    <hyperlink ref="E26" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
-    <hyperlink ref="E18" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
-    <hyperlink ref="E22" r:id="rId20" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
-    <hyperlink ref="E28" r:id="rId21" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
-    <hyperlink ref="E27" r:id="rId22" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
-    <hyperlink ref="F10" r:id="rId23" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
-    <hyperlink ref="E13" r:id="rId24" xr:uid="{CBA56252-7528-480E-896E-AE82E42DF951}"/>
-    <hyperlink ref="E16" r:id="rId25" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
-    <hyperlink ref="E15" r:id="rId26" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="E12" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="E11" r:id="rId28" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
-    <hyperlink ref="E7" r:id="rId29" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
-    <hyperlink ref="E3" r:id="rId30" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="F6" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="E26" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="E24" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="E18" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="E20" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="E22" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="E21" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="E25" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="E27" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="E19" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="E23" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="E29" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="E28" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="F11" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="E14" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="E17" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="E16" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="E13" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="E12" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
+    <hyperlink ref="E7" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
+    <hyperlink ref="E3" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
+    <hyperlink ref="E8" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
phd current data an home no.of data update
</commit_message>
<xml_diff>
--- a/excels/Phd_Current.xlsx
+++ b/excels/Phd_Current.xlsx
@@ -1,16 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\nitw\NITW-Transportation-Division\excels\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{075FE5DC-FE3B-4F62-9377-552FC44D2039}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView windowWidth="22188" windowHeight="9000"/>
   </bookViews>
   <sheets>
     <sheet name="Rs" sheetId="1" r:id="rId1"/>
@@ -36,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="188">
   <si>
     <t xml:space="preserve">Name </t>
   </si>
@@ -375,6 +369,9 @@
   </si>
   <si>
     <t>kd25cer2p03@student.nitw.ac.in</t>
+  </si>
+  <si>
+    <t>Phd_Current/25CER2P03</t>
   </si>
   <si>
     <t>Lohit Havalagi</t>
@@ -602,8 +599,14 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="17">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="4">
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ &quot;₹&quot;* #,##0.00_ ;_ &quot;₹&quot;* \-#,##0.00_ ;_ &quot;₹&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="36">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -714,16 +717,345 @@
       <name val="Times New Roman "/>
       <charset val="134"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="33">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -731,12 +1063,251 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="176" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -747,11 +1318,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -764,21 +1336,24 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="6"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -786,20 +1361,63 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="6" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
+    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
+    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
+    <cellStyle name="Note" xfId="8" builtinId="10"/>
+    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
+    <cellStyle name="Title" xfId="10" builtinId="15"/>
+    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
+    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
+    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
+    <cellStyle name="Input" xfId="16" builtinId="20"/>
+    <cellStyle name="Output" xfId="17" builtinId="21"/>
+    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
+    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
+    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
+    <cellStyle name="Total" xfId="21" builtinId="25"/>
+    <cellStyle name="Good" xfId="22" builtinId="26"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
+    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
+    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
+    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1057,27 +1675,27 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:H44"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.6" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="29.140625" customWidth="1"/>
+    <col min="1" max="1" width="29.1388888888889" customWidth="1"/>
     <col min="2" max="2" width="22" style="1" customWidth="1"/>
-    <col min="3" max="3" width="19.42578125" customWidth="1"/>
-    <col min="4" max="4" width="69.28515625" customWidth="1"/>
-    <col min="5" max="5" width="57.5703125" style="2" customWidth="1"/>
-    <col min="6" max="6" width="42.7109375" customWidth="1"/>
-    <col min="7" max="7" width="86.28515625" customWidth="1"/>
-    <col min="10" max="10" width="33.7109375" customWidth="1"/>
-    <col min="11" max="11" width="22.28515625" customWidth="1"/>
+    <col min="3" max="3" width="19.4259259259259" customWidth="1"/>
+    <col min="4" max="4" width="69.287037037037" customWidth="1"/>
+    <col min="5" max="5" width="57.5740740740741" style="2" customWidth="1"/>
+    <col min="6" max="6" width="42.712962962963" customWidth="1"/>
+    <col min="7" max="7" width="86.287037037037" customWidth="1"/>
+    <col min="10" max="10" width="33.712962962963" customWidth="1"/>
+    <col min="11" max="11" width="22.287037037037" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="16.5">
+    <row r="1" spans="1:8">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1103,1033 +1721,1036 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="16.5">
+    <row r="2" spans="1:8">
       <c r="A2" s="6" t="s">
         <v>8</v>
       </c>
       <c r="B2" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="6">
+      <c r="C2" s="8">
         <v>9494353643</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="8" t="s">
         <v>10</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F2" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="8" t="s">
+      <c r="G2" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="H2" s="8" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="16.5">
+    <row r="3" spans="1:8">
       <c r="A3" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B3" s="7">
         <v>720028</v>
       </c>
-      <c r="C3" s="6">
+      <c r="C3" s="8">
         <v>8296368016</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="G3" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="H3" s="8" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="16.5">
+    <row r="4" spans="1:8">
       <c r="A4" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="11">
         <v>9492203336</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="11" t="s">
+      <c r="E4" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="F4" s="12" t="s">
+      <c r="F4" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="G4" s="13" t="s">
+      <c r="G4" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="H4" s="8" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="16.5">
-      <c r="A5" s="14" t="s">
+    <row r="5" spans="1:8">
+      <c r="A5" s="15" t="s">
         <v>26</v>
       </c>
       <c r="B5" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="8">
         <v>7902240230</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="8" t="s">
         <v>28</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="F5" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="G5" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="H5" s="8" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="16.5">
-      <c r="A6" s="14" t="s">
+    <row r="6" spans="1:8">
+      <c r="A6" s="15" t="s">
         <v>32</v>
       </c>
       <c r="B6" s="7">
         <v>712029</v>
       </c>
-      <c r="C6" s="6">
+      <c r="C6" s="8">
         <v>9652055481</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="8" t="s">
         <v>33</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="F6" s="15" t="s">
+      <c r="F6" s="16" t="s">
         <v>35</v>
       </c>
-      <c r="G6" s="14" t="s">
+      <c r="G6" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="H6" s="6" t="s">
+      <c r="H6" s="8" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="16.5">
-      <c r="A7" s="14" t="s">
+    <row r="7" spans="1:8">
+      <c r="A7" s="15" t="s">
         <v>37</v>
       </c>
       <c r="B7" s="7">
         <v>720010</v>
       </c>
-      <c r="C7" s="6">
+      <c r="C7" s="8">
         <v>9704634125</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="8" t="s">
         <v>28</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="F7" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="G7" s="14" t="s">
+      <c r="G7" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="H7" s="6" t="s">
+      <c r="H7" s="8" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="16.5">
-      <c r="A8" s="14" t="s">
+    <row r="8" spans="1:8">
+      <c r="A8" s="15" t="s">
         <v>41</v>
       </c>
       <c r="B8" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C8" s="6">
+      <c r="C8" s="8">
         <v>9790986371</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="F8" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="G8" s="16" t="s">
+      <c r="G8" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="H8" s="6" t="s">
+      <c r="H8" s="8" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="16.5">
+    <row r="9" spans="1:8">
       <c r="A9" s="6" t="s">
         <v>46</v>
       </c>
       <c r="B9" s="7">
         <v>720029</v>
       </c>
-      <c r="C9" s="6">
+      <c r="C9" s="8">
         <v>7296367016</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="F9" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="G9" s="6" t="s">
+      <c r="G9" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="H9" s="6" t="s">
+      <c r="H9" s="8" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="16.5">
+    <row r="10" spans="1:8">
       <c r="A10" s="6" t="s">
         <v>49</v>
       </c>
       <c r="B10" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="C10" s="6">
+      <c r="C10" s="8">
         <v>9495307599</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="E10" s="17" t="s">
+      <c r="E10" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="F10" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="G10" s="6" t="s">
+      <c r="G10" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="H10" s="6" t="s">
+      <c r="H10" s="8" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="16.5">
+    <row r="11" spans="1:8">
       <c r="A11" s="6" t="s">
         <v>54</v>
       </c>
       <c r="B11" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="C11" s="6">
+      <c r="C11" s="8">
         <v>9167519065</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D11" s="8" t="s">
         <v>56</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="F11" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="G11" s="6" t="s">
+      <c r="G11" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="H11" s="6" t="s">
+      <c r="H11" s="8" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="16.5">
+    <row r="12" spans="1:8">
       <c r="A12" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="C12" s="12">
+      <c r="C12" s="13">
         <v>8500970790</v>
       </c>
-      <c r="D12" s="12" t="s">
+      <c r="D12" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="E12" s="11" t="s">
+      <c r="E12" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="F12" s="6" t="s">
+      <c r="F12" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="G12" s="13" t="s">
+      <c r="G12" s="14" t="s">
         <v>65</v>
       </c>
-      <c r="H12" s="6" t="s">
+      <c r="H12" s="8" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="16.5">
+    <row r="13" spans="1:8">
       <c r="A13" s="6" t="s">
         <v>66</v>
       </c>
       <c r="B13" s="7">
         <v>720030</v>
       </c>
-      <c r="C13" s="6">
+      <c r="C13" s="8">
         <v>6296367016</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="D13" s="8" t="s">
         <v>67</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="F13" s="8" t="s">
+      <c r="F13" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="G13" s="18" t="s">
+      <c r="G13" s="20" t="s">
         <v>69</v>
       </c>
-      <c r="H13" s="6" t="s">
+      <c r="H13" s="8" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="16.5">
+    <row r="14" spans="1:8">
       <c r="A14" s="6" t="s">
         <v>70</v>
       </c>
       <c r="B14" s="7">
         <v>720019</v>
       </c>
-      <c r="C14" s="6">
+      <c r="C14" s="8">
         <v>7386310538</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="D14" s="8" t="s">
         <v>10</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="F14" s="8" t="s">
+      <c r="F14" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="G14" s="18" t="s">
+      <c r="G14" s="20" t="s">
         <v>73</v>
       </c>
-      <c r="H14" s="6" t="s">
+      <c r="H14" s="8" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="16.5">
+    <row r="15" spans="1:8">
       <c r="A15" s="6" t="s">
         <v>74</v>
       </c>
       <c r="B15" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="C15" s="6">
+      <c r="C15" s="8">
         <v>9989981013</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="D15" s="8" t="s">
         <v>33</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="F15" s="15" t="s">
+      <c r="F15" s="16" t="s">
         <v>77</v>
       </c>
       <c r="G15" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="H15" s="6" t="s">
+      <c r="H15" s="8" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="16.5">
+    <row r="16" spans="1:8">
       <c r="A16" s="6" t="s">
         <v>79</v>
       </c>
       <c r="B16" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="C16" s="6">
+      <c r="C16" s="8">
         <v>9951815536</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="D16" s="8" t="s">
         <v>33</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="F16" s="8" t="s">
+      <c r="F16" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="G16" s="6" t="s">
+      <c r="G16" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="H16" s="6" t="s">
+      <c r="H16" s="8" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="16.5">
+    <row r="17" spans="1:8">
       <c r="A17" s="6" t="s">
         <v>84</v>
       </c>
       <c r="B17" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="D17" s="6" t="s">
+      <c r="D17" s="8" t="s">
         <v>62</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="F17" s="15" t="s">
+      <c r="F17" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="G17" s="6" t="s">
+      <c r="G17" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="H17" s="6" t="s">
+      <c r="H17" s="8" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="16.5">
+    <row r="18" spans="1:8">
       <c r="A18" s="6" t="s">
         <v>90</v>
       </c>
       <c r="B18" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="C18" s="6">
+      <c r="C18" s="8">
         <v>9542093078</v>
       </c>
-      <c r="D18" s="6" t="s">
+      <c r="D18" s="8" t="s">
         <v>92</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="F18" s="13" t="s">
+      <c r="F18" s="14" t="s">
         <v>94</v>
       </c>
-      <c r="G18" s="6" t="s">
+      <c r="G18" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="H18" s="6" t="s">
+      <c r="H18" s="8" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="16.5">
+    <row r="19" spans="1:8">
       <c r="A19" s="6" t="s">
         <v>96</v>
       </c>
       <c r="B19" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="C19" s="6">
+      <c r="C19" s="8">
         <v>7702907803</v>
       </c>
-      <c r="D19" s="6" t="s">
+      <c r="D19" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="F19" s="13" t="s">
+      <c r="F19" s="14" t="s">
         <v>98</v>
       </c>
-      <c r="G19" s="6" t="s">
+      <c r="G19" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="H19" s="6" t="s">
+      <c r="H19" s="8" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="16.5">
+    <row r="20" spans="1:8">
       <c r="A20" s="6" t="s">
         <v>100</v>
       </c>
       <c r="B20" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="C20" s="6">
+      <c r="C20" s="8">
         <v>9381442621</v>
       </c>
-      <c r="D20" s="6" t="s">
+      <c r="D20" s="8" t="s">
         <v>10</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="F20" s="8" t="s">
+      <c r="F20" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="G20" s="6" t="s">
+      <c r="G20" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="H20" s="6" t="s">
+      <c r="H20" s="8" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="16.5">
+    <row r="21" spans="1:8">
       <c r="A21" s="6" t="s">
         <v>104</v>
       </c>
       <c r="B21" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="C21" s="6">
+      <c r="C21" s="8">
         <v>8639717077</v>
       </c>
-      <c r="D21" s="6" t="s">
+      <c r="D21" s="8" t="s">
         <v>10</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="F21" s="8" t="s">
+      <c r="F21" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="G21" s="6" t="s">
+      <c r="G21" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="H21" s="6" t="s">
+      <c r="H21" s="8" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="16.5">
+    <row r="22" spans="1:8">
       <c r="A22" s="6" t="s">
         <v>109</v>
       </c>
       <c r="B22" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="C22" s="6">
+      <c r="C22" s="8">
         <v>6396421104</v>
       </c>
-      <c r="D22" s="6" t="s">
+      <c r="D22" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="F22" s="8" t="s">
+      <c r="F22" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="G22" s="6"/>
-      <c r="H22" s="6" t="s">
+      <c r="G22" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="H22" s="8" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="16.5">
+    <row r="23" spans="1:8">
       <c r="A23" s="6" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>114</v>
-      </c>
-      <c r="C23" s="6">
+        <v>115</v>
+      </c>
+      <c r="C23" s="8">
         <v>8296369017</v>
       </c>
-      <c r="D23" s="6" t="s">
-        <v>115</v>
+      <c r="D23" s="8" t="s">
+        <v>116</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="F23" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="F23" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="G23" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="H23" s="6" t="s">
+      <c r="G23" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="H23" s="8" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="16.5">
+    <row r="24" spans="1:8">
       <c r="A24" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="C24" s="6">
+        <v>120</v>
+      </c>
+      <c r="C24" s="8">
         <v>8008584329</v>
       </c>
-      <c r="D24" s="6" t="s">
+      <c r="D24" s="8" t="s">
         <v>28</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="F24" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="G24" s="6" t="s">
+      <c r="F24" s="16" t="s">
         <v>122</v>
       </c>
-      <c r="H24" s="6" t="s">
+      <c r="G24" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="H24" s="8" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="16.5">
+    <row r="25" spans="1:8">
       <c r="A25" s="6" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>124</v>
-      </c>
-      <c r="C25" s="6">
+        <v>125</v>
+      </c>
+      <c r="C25" s="8">
         <v>9032426878</v>
       </c>
-      <c r="D25" s="6" t="s">
+      <c r="D25" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="F25" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="G25" s="8" t="s">
+      <c r="F25" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="H25" s="6" t="s">
+      <c r="G25" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="H25" s="8" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="16.5">
+    <row r="26" spans="1:8">
       <c r="A26" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>129</v>
-      </c>
-      <c r="C26" s="6">
+        <v>130</v>
+      </c>
+      <c r="C26" s="8">
         <v>8296369016</v>
       </c>
-      <c r="D26" s="6" t="s">
+      <c r="D26" s="8" t="s">
         <v>10</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="F26" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="F26" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="G26" s="6" t="s">
-        <v>131</v>
-      </c>
-      <c r="H26" s="6" t="s">
+      <c r="G26" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="H26" s="8" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="16.5">
+    <row r="27" spans="1:8">
       <c r="A27" s="6" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>133</v>
-      </c>
-      <c r="C27" s="6">
+        <v>134</v>
+      </c>
+      <c r="C27" s="8">
         <v>8121007701</v>
       </c>
-      <c r="D27" s="6" t="s">
+      <c r="D27" s="8" t="s">
         <v>28</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="F27" s="15" t="s">
         <v>135</v>
       </c>
-      <c r="G27" s="6" t="s">
+      <c r="F27" s="16" t="s">
         <v>136</v>
       </c>
-      <c r="H27" s="6" t="s">
+      <c r="G27" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="H27" s="8" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="16.5">
+    <row r="28" spans="1:8">
       <c r="A28" s="6" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="C28" s="6">
+        <v>139</v>
+      </c>
+      <c r="C28" s="8">
         <v>8236367016</v>
       </c>
-      <c r="D28" s="6" t="s">
+      <c r="D28" s="8" t="s">
         <v>10</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="F28" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="F28" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="G28" s="6" t="s">
-        <v>140</v>
-      </c>
-      <c r="H28" s="6" t="s">
+      <c r="G28" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="H28" s="8" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="16.5">
+    <row r="29" spans="1:8">
       <c r="A29" s="6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B29" s="7">
         <v>720021</v>
       </c>
-      <c r="C29" s="6">
+      <c r="C29" s="8">
         <v>9866886438</v>
       </c>
-      <c r="D29" s="6" t="s">
+      <c r="D29" s="8" t="s">
         <v>10</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="F29" s="15" t="s">
         <v>143</v>
       </c>
-      <c r="G29" s="18" t="s">
+      <c r="F29" s="16" t="s">
         <v>144</v>
       </c>
-      <c r="H29" s="6" t="s">
+      <c r="G29" s="20" t="s">
+        <v>145</v>
+      </c>
+      <c r="H29" s="8" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="16.5">
+    <row r="30" spans="1:8">
       <c r="A30" s="6" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B30" s="7">
         <v>720032</v>
       </c>
-      <c r="C30" s="6">
+      <c r="C30" s="8">
         <v>9296367016</v>
       </c>
-      <c r="D30" s="6" t="s">
+      <c r="D30" s="8" t="s">
         <v>10</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="F30" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="F30" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="G30" s="18" t="s">
-        <v>147</v>
-      </c>
-      <c r="H30" s="6" t="s">
+      <c r="G30" s="20" t="s">
+        <v>148</v>
+      </c>
+      <c r="H30" s="8" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="18.75">
+    <row r="31" ht="18" spans="1:8">
       <c r="A31" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="B31" s="19">
+        <v>149</v>
+      </c>
+      <c r="B31" s="21">
         <v>720027</v>
       </c>
-      <c r="C31" s="20">
+      <c r="C31" s="22">
         <v>7893754499</v>
       </c>
-      <c r="D31" s="6" t="s">
+      <c r="D31" s="8" t="s">
         <v>10</v>
       </c>
       <c r="E31" t="s">
         <v>23</v>
       </c>
-      <c r="F31" s="21" t="s">
-        <v>149</v>
+      <c r="F31" s="23" t="s">
+        <v>150</v>
       </c>
       <c r="G31" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="H31" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="H31" s="8" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="16.5">
-      <c r="A32" s="22" t="s">
-        <v>151</v>
+    <row r="32" spans="1:8">
+      <c r="A32" s="24" t="s">
+        <v>152</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>152</v>
-      </c>
-      <c r="C32" s="6">
+        <v>153</v>
+      </c>
+      <c r="C32" s="8">
         <v>9505306946</v>
       </c>
-      <c r="D32" s="6" t="s">
+      <c r="D32" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="F32" s="8" t="s">
-        <v>153</v>
-      </c>
-      <c r="G32" s="18" t="s">
+      <c r="F32" s="9" t="s">
         <v>154</v>
       </c>
-      <c r="H32" s="6" t="s">
+      <c r="G32" s="20" t="s">
+        <v>155</v>
+      </c>
+      <c r="H32" s="8" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="16.5">
+    <row r="33" spans="1:8">
       <c r="A33" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>156</v>
-      </c>
-      <c r="C33" s="6">
+        <v>157</v>
+      </c>
+      <c r="C33" s="8">
         <v>9381752788</v>
       </c>
-      <c r="D33" s="6" t="s">
+      <c r="D33" s="8" t="s">
         <v>62</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="F33" s="8" t="s">
         <v>158</v>
       </c>
-      <c r="G33" s="6" t="s">
+      <c r="F33" s="9" t="s">
         <v>159</v>
       </c>
-      <c r="H33" s="6" t="s">
+      <c r="G33" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="H33" s="8" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="16.5">
+    <row r="34" spans="1:8">
       <c r="A34" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>161</v>
-      </c>
-      <c r="C34" s="6">
+        <v>162</v>
+      </c>
+      <c r="C34" s="8">
         <v>9149344247</v>
       </c>
-      <c r="D34" s="6" t="s">
-        <v>162</v>
+      <c r="D34" s="8" t="s">
+        <v>163</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="F34" s="8" t="s">
         <v>164</v>
       </c>
-      <c r="G34" s="6" t="s">
+      <c r="F34" s="9" t="s">
         <v>165</v>
       </c>
-      <c r="H34" s="6" t="s">
+      <c r="G34" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="H34" s="8" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="16.5">
+    <row r="35" spans="1:8">
       <c r="A35" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B35" s="7">
         <v>720026</v>
       </c>
-      <c r="C35" s="6">
+      <c r="C35" s="8">
         <v>8196367016</v>
       </c>
-      <c r="D35" s="6" t="s">
+      <c r="D35" s="8" t="s">
         <v>10</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="F35" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="F35" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="G35" s="18" t="s">
-        <v>168</v>
-      </c>
-      <c r="H35" s="6" t="s">
+      <c r="G35" s="20" t="s">
+        <v>169</v>
+      </c>
+      <c r="H35" s="8" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="16.5">
+    <row r="36" spans="1:8">
       <c r="A36" s="6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B36" s="7">
         <v>720018</v>
       </c>
-      <c r="C36" s="23">
+      <c r="C36" s="25">
         <v>9555541646</v>
       </c>
-      <c r="D36" s="23" t="s">
+      <c r="D36" s="25" t="s">
         <v>62</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="F36" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="G36" s="6" t="s">
+      <c r="F36" s="9" t="s">
         <v>172</v>
       </c>
-      <c r="H36" s="6" t="s">
+      <c r="G36" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="H36" s="8" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="16.5">
+    <row r="37" spans="1:8">
       <c r="A37" s="6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>174</v>
-      </c>
-      <c r="C37" s="6">
+        <v>175</v>
+      </c>
+      <c r="C37" s="8">
         <v>8296367116</v>
       </c>
-      <c r="D37" s="6" t="s">
+      <c r="D37" s="8" t="s">
         <v>10</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="F37" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="F37" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="G37" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="H37" s="6" t="s">
+      <c r="G37" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="H37" s="8" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="16.5">
+    <row r="38" spans="1:8">
       <c r="A38" s="6" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>178</v>
-      </c>
-      <c r="C38" s="6">
+        <v>179</v>
+      </c>
+      <c r="C38" s="8">
         <v>8286367016</v>
       </c>
-      <c r="D38" s="6" t="s">
-        <v>179</v>
+      <c r="D38" s="8" t="s">
+        <v>180</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="F38" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="F38" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="G38" s="8" t="s">
-        <v>181</v>
-      </c>
-      <c r="H38" s="6" t="s">
+      <c r="G38" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="H38" s="8" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="39" spans="1:8" ht="16.5">
+    <row r="39" spans="1:8">
       <c r="A39" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>183</v>
-      </c>
-      <c r="C39" s="6">
+        <v>184</v>
+      </c>
+      <c r="C39" s="8">
         <v>9948673907</v>
       </c>
-      <c r="D39" s="6" t="s">
+      <c r="D39" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="F39" s="8" t="s">
         <v>185</v>
       </c>
-      <c r="G39" s="8" t="s">
+      <c r="F39" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="H39" s="6" t="s">
+      <c r="G39" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="H39" s="8" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="16.5">
-      <c r="A40" s="24"/>
-      <c r="B40" s="25"/>
-      <c r="C40" s="26"/>
-      <c r="D40" s="26"/>
-      <c r="E40" s="17"/>
-      <c r="F40" s="27"/>
-      <c r="G40" s="26"/>
-      <c r="H40" s="26"/>
-    </row>
-    <row r="44" spans="1:8" ht="16.5">
-      <c r="G44" s="6"/>
+    <row r="40" spans="1:8">
+      <c r="A40" s="26"/>
+      <c r="B40" s="27"/>
+      <c r="C40" s="28"/>
+      <c r="D40" s="28"/>
+      <c r="E40" s="19"/>
+      <c r="F40" s="29"/>
+      <c r="G40" s="28"/>
+      <c r="H40" s="28"/>
+    </row>
+    <row r="44" spans="1:8">
+      <c r="G44" s="8"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G27">
-    <sortCondition ref="A12:A27"/>
+  <sortState ref="A2:G28">
+    <sortCondition ref="A12:A28"/>
   </sortState>
   <hyperlinks>
-    <hyperlink ref="F11" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="F18" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="G12" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="G4" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="F2" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="F5" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="G5" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="G2" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="F36" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="F33" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="F23" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="F26" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="F28" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="F35" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="F37" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
-    <hyperlink ref="F25" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="F30" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="F39" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="F38" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="F16" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
-    <hyperlink ref="F21" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
-    <hyperlink ref="F20" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
-    <hyperlink ref="F14" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
-    <hyperlink ref="F13" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
-    <hyperlink ref="F9" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
-    <hyperlink ref="F3" r:id="rId26" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
-    <hyperlink ref="F10" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
-    <hyperlink ref="F6" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
-    <hyperlink ref="F15" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
-    <hyperlink ref="F31" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
-    <hyperlink ref="F29" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
-    <hyperlink ref="F27" r:id="rId32" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
-    <hyperlink ref="F24" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
-    <hyperlink ref="F17" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
+    <hyperlink ref="F11" r:id="rId1" display="bd22cer2r11@student.nitw.ac.in"/>
+    <hyperlink ref="F18" r:id="rId2" display="gd21cerer15@student.nitw.ac.in"/>
+    <hyperlink ref="G12" r:id="rId3" display="https://www.nitw.ac.in/CIVDeptAssets/images/phd86.jpg"/>
+    <hyperlink ref="G4" r:id="rId4" display="https://www.nitw.ac.in/CIVDeptAssets/images/phd126.jpg"/>
+    <hyperlink ref="F2" r:id="rId5" display="ab23cer2r10@student.nitw.ac.in"/>
+    <hyperlink ref="F5" r:id="rId6" display="aa23cer1r01@student.nitw.ac.in"/>
+    <hyperlink ref="G5" r:id="rId7" display="https://nitw.ac.in/api/static/files/Anusree_A_2025-6-19-10-53-48.jpg"/>
+    <hyperlink ref="G2" r:id="rId8" display="https://nitw.ac.in/api/static/files/Aenugu_Bharadwaj_2025-6-19-10-52-15.jpg"/>
+    <hyperlink ref="F36" r:id="rId9" display="ckumarcivil@gmail.com"/>
+    <hyperlink ref="F33" r:id="rId10" display="bs25cer2r13@student.nitw.ac.in"/>
+    <hyperlink ref="F23" r:id="rId5" display="ab23cer2r10@student.nitw.ac.in"/>
+    <hyperlink ref="F26" r:id="rId5" display="ab23cer2r10@student.nitw.ac.in"/>
+    <hyperlink ref="F28" r:id="rId5" display="ab23cer2r10@student.nitw.ac.in"/>
+    <hyperlink ref="F35" r:id="rId5" display="ab23cer2r10@student.nitw.ac.in"/>
+    <hyperlink ref="F37" r:id="rId5" display="ab23cer2r10@student.nitw.ac.in"/>
+    <hyperlink ref="F25" r:id="rId11" display="ma25cer2r10@student.nitw.ac.in"/>
+    <hyperlink ref="F30" r:id="rId5" display="ab23cer2r10@student.nitw.ac.in"/>
+    <hyperlink ref="F39" r:id="rId12" display="yp25cer2r08@student.nitw.ac.in"/>
+    <hyperlink ref="F38" r:id="rId5" display="ab23cer2r10@student.nitw.ac.in"/>
+    <hyperlink ref="F16" r:id="rId13" display="gm25cer1r08@student.nitw.ac.in"/>
+    <hyperlink ref="F21" r:id="rId14" display="ab25cer2r10@student.nitw.ac.in"/>
+    <hyperlink ref="F20" r:id="rId5" display="ab23cer2r10@student.nitw.ac.in"/>
+    <hyperlink ref="F14" r:id="rId15" display="ab24cer2r10@student.nitw.ac.in"/>
+    <hyperlink ref="F13" r:id="rId5" display="ab23cer2r10@student.nitw.ac.in"/>
+    <hyperlink ref="F9" r:id="rId5" display="ab23cer2r10@student.nitw.ac.in"/>
+    <hyperlink ref="F3" r:id="rId5" display="ab23cer2r10@student.nitw.ac.in"/>
+    <hyperlink ref="F10" r:id="rId16" display="ab22cer2p01@student.nitw.ac.in"/>
+    <hyperlink ref="F6" r:id="rId17" display="br712029@student.nitw.ac.in"/>
+    <hyperlink ref="F15" r:id="rId18" display="gv23cer2p06@student.nitw.ac.in"/>
+    <hyperlink ref="F31" r:id="rId19" display="rr720027@student.nitw.ac.in"/>
+    <hyperlink ref="F29" r:id="rId20" display="dhatrikalyan@gmail.com"/>
+    <hyperlink ref="F27" r:id="rId21" display="np26cer1r11@student.nitw.ac.in "/>
+    <hyperlink ref="F24" r:id="rId22" display="ms26cer1r04@student.nitw.ac.in "/>
+    <hyperlink ref="F17" r:id="rId23" display="gs26cer1r02@student.nitw.ac.in"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>